<commit_message>
data(fate-star-rail-night): G19-P4-B2 execute semantic fixtures
</commit_message>
<xml_diff>
--- a/config/fate-star-rail-night/data/FateStarRailNight.xlsx
+++ b/config/fate-star-rail-night/data/FateStarRailNight.xlsx
@@ -1224,7 +1224,7 @@
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>[{"locator":"root","path":"content-reference/fate-star-rail-night-v1/pack-index.json","sha256":"ae040b74b3fddbb7e59807a435017311ec91e5892e364430636d25123bb7ecc3"}]</t>
+          <t>[{"locator":"root","path":"content-reference/fate-star-rail-night-v1/pack-index.json","sha256":"3a931ae76149992b513fd7c1ff819a55225baa8e99c8530bc343338340854018"}]</t>
         </is>
       </c>
       <c r="M8" s="11" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="Q8" s="11" t="inlineStr">
         <is>
-          <t>{"manifest_obligations":"undefined","normalized_records":"2018","pack_sha256":"ae040b74b3fddbb7e59807a435017311ec91e5892e364430636d25123bb7ecc3","runtime_executable":"false"}</t>
+          <t>{"manifest_obligations":"undefined","normalized_records":"2018","pack_sha256":"3a931ae76149992b513fd7c1ff819a55225baa8e99c8530bc343338340854018","runtime_executable":"false"}</t>
         </is>
       </c>
       <c r="R8" s="11" t="inlineStr">

</xml_diff>

<commit_message>
data(fate-star-rail-night): G19-P4-B3 reconcile peer manifests
</commit_message>
<xml_diff>
--- a/config/fate-star-rail-night/data/FateStarRailNight.xlsx
+++ b/config/fate-star-rail-night/data/FateStarRailNight.xlsx
@@ -1224,7 +1224,7 @@
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>[{"locator":"root","path":"content-reference/fate-star-rail-night-v1/pack-index.json","sha256":"3a931ae76149992b513fd7c1ff819a55225baa8e99c8530bc343338340854018"}]</t>
+          <t>[{"locator":"root","path":"content-reference/fate-star-rail-night-v1/pack-index.json","sha256":"59bcb142e1d7be2b95f6a99ba3ad806f1afefa8ce8708066591b08bc51aa171d"}]</t>
         </is>
       </c>
       <c r="M8" s="11" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="Q8" s="11" t="inlineStr">
         <is>
-          <t>{"manifest_obligations":"undefined","normalized_records":"2018","pack_sha256":"3a931ae76149992b513fd7c1ff819a55225baa8e99c8530bc343338340854018","runtime_executable":"false"}</t>
+          <t>{"manifest_obligations":"undefined","normalized_records":"2018","pack_sha256":"59bcb142e1d7be2b95f6a99ba3ad806f1afefa8ce8708066591b08bc51aa171d","runtime_executable":"false"}</t>
         </is>
       </c>
       <c r="R8" s="11" t="inlineStr">

</xml_diff>